<commit_message>
Fixed TOF Results obtained
</commit_message>
<xml_diff>
--- a/Pastas_Mortero_2025/Plantilla_RESULTADOS_CPT (072025).xlsx
+++ b/Pastas_Mortero_2025/Plantilla_RESULTADOS_CPT (072025).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariajosetorresconstante/Documents/GitHub/SingleSolitaryWaveAnalysis/Pastas_Mortero_2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470C9D44-A29C-E14F-9861-CE05E80F4118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FD087DA-5375-5E40-9A82-5DC093B38C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{6AC846BB-F0A6-40EE-9D25-7222205E4360}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16080" activeTab="1" xr2:uid="{6AC846BB-F0A6-40EE-9D25-7222205E4360}"/>
   </bookViews>
   <sheets>
     <sheet name="CPT" sheetId="1" r:id="rId1"/>
@@ -922,7 +922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1011,6 +1011,23 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1050,29 +1067,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2873,7 +2870,7 @@
                   <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="es-EC"/>
+              <a:endParaRPr lang="es-MX"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3123,6 +3120,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="342460800"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -7859,10 +7857,10 @@
       <c r="N1" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="83" t="s">
+      <c r="O1" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="84"/>
+      <c r="P1" s="91"/>
     </row>
     <row r="2" spans="1:24" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="17" t="s">
@@ -7905,10 +7903,10 @@
       <c r="N2" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="85" t="s">
+      <c r="O2" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="P2" s="86"/>
+      <c r="P2" s="93"/>
     </row>
     <row r="3" spans="1:24" ht="19" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
@@ -7949,10 +7947,10 @@
       <c r="N3" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="87" t="s">
+      <c r="O3" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="P3" s="88"/>
+      <c r="P3" s="95"/>
     </row>
     <row r="4" spans="1:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
@@ -7965,39 +7963,39 @@
       <c r="A5" s="60">
         <v>45853</v>
       </c>
-      <c r="B5" s="76" t="s">
+      <c r="B5" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="77"/>
-      <c r="D5" s="77"/>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
+      <c r="C5" s="84"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
       <c r="I5" s="61">
         <v>45853</v>
       </c>
-      <c r="J5" s="78" t="s">
+      <c r="J5" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="78"/>
-      <c r="L5" s="78"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="78"/>
-      <c r="O5" s="78"/>
-      <c r="P5" s="79"/>
+      <c r="K5" s="85"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="85"/>
+      <c r="O5" s="85"/>
+      <c r="P5" s="86"/>
       <c r="Q5" s="62">
         <v>45853</v>
       </c>
-      <c r="R5" s="80" t="s">
+      <c r="R5" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="S5" s="81"/>
-      <c r="T5" s="81"/>
-      <c r="U5" s="81"/>
-      <c r="V5" s="81"/>
-      <c r="W5" s="81"/>
-      <c r="X5" s="82"/>
+      <c r="S5" s="88"/>
+      <c r="T5" s="88"/>
+      <c r="U5" s="88"/>
+      <c r="V5" s="88"/>
+      <c r="W5" s="88"/>
+      <c r="X5" s="89"/>
     </row>
     <row r="6" spans="1:24" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
@@ -8753,326 +8751,326 @@
       </c>
       <c r="C3" s="96"/>
       <c r="D3" s="96"/>
-      <c r="E3" s="97"/>
+      <c r="E3" s="82"/>
       <c r="F3" s="96">
         <v>0.35</v>
       </c>
       <c r="G3" s="96"/>
       <c r="H3" s="96"/>
-      <c r="I3" s="97"/>
-      <c r="J3" s="98">
+      <c r="I3" s="82"/>
+      <c r="J3" s="97">
         <v>0.4</v>
       </c>
-      <c r="K3" s="98"/>
-      <c r="L3" s="98"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B4" s="89"/>
-      <c r="C4" s="89" t="s">
+      <c r="B4" s="76"/>
+      <c r="C4" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="89" t="s">
+      <c r="D4" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="89"/>
-      <c r="G4" s="89" t="s">
+      <c r="F4" s="76"/>
+      <c r="G4" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="89" t="s">
+      <c r="H4" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92" t="s">
+      <c r="J4" s="79"/>
+      <c r="K4" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="92" t="s">
+      <c r="L4" s="79" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B5" s="89">
+      <c r="B5" s="76">
         <v>0</v>
       </c>
-      <c r="C5" s="90">
+      <c r="C5" s="77">
         <v>25.166666666666668</v>
       </c>
-      <c r="D5" s="89">
+      <c r="D5" s="76">
         <v>3.188538838648558E-3</v>
       </c>
-      <c r="F5" s="89">
+      <c r="F5" s="76">
         <v>0</v>
       </c>
-      <c r="G5" s="91">
+      <c r="G5" s="78">
         <v>39.700000000000003</v>
       </c>
-      <c r="H5" s="89">
+      <c r="H5" s="76">
         <v>3.5987030996700309E-3</v>
       </c>
-      <c r="J5" s="92">
+      <c r="J5" s="79">
         <v>0</v>
       </c>
-      <c r="K5" s="93">
+      <c r="K5" s="80">
         <v>39.5</v>
       </c>
-      <c r="L5" s="92">
+      <c r="L5" s="79">
         <v>3.541735841195178E-3</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B6" s="89">
+      <c r="B6" s="76">
         <v>5</v>
       </c>
-      <c r="C6" s="90">
+      <c r="C6" s="77">
         <v>24.599999999999998</v>
       </c>
-      <c r="D6" s="89">
+      <c r="D6" s="76">
         <v>2.8237158649864519E-3</v>
       </c>
-      <c r="F6" s="89">
+      <c r="F6" s="76">
         <v>5</v>
       </c>
-      <c r="G6" s="91">
+      <c r="G6" s="78">
         <v>39.700000000000003</v>
       </c>
-      <c r="H6" s="89">
+      <c r="H6" s="76">
         <v>3.649624853164684E-3</v>
       </c>
-      <c r="J6" s="92">
+      <c r="J6" s="79">
         <v>5</v>
       </c>
-      <c r="K6" s="93">
+      <c r="K6" s="80">
         <v>39.5</v>
       </c>
-      <c r="L6" s="92">
+      <c r="L6" s="79">
         <v>4.1146636978582523E-3</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B7" s="89">
+      <c r="B7" s="76">
         <v>10</v>
       </c>
-      <c r="C7" s="90">
+      <c r="C7" s="77">
         <v>20.166666666666668</v>
       </c>
-      <c r="D7" s="89">
+      <c r="D7" s="76">
         <v>2.832086564190206E-3</v>
       </c>
-      <c r="F7" s="89">
+      <c r="F7" s="76">
         <v>10</v>
       </c>
-      <c r="G7" s="91">
+      <c r="G7" s="78">
         <v>39.700000000000003</v>
       </c>
-      <c r="H7" s="89">
+      <c r="H7" s="76">
         <v>3.9872430544117977E-3</v>
       </c>
-      <c r="J7" s="92">
+      <c r="J7" s="79">
         <v>10</v>
       </c>
-      <c r="K7" s="93">
+      <c r="K7" s="80">
         <v>39.5</v>
       </c>
-      <c r="L7" s="92">
+      <c r="L7" s="79">
         <v>4.1741886699789687E-3</v>
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B8" s="89">
+      <c r="B8" s="76">
         <v>20</v>
       </c>
-      <c r="C8" s="90">
+      <c r="C8" s="77">
         <v>20.2</v>
       </c>
-      <c r="D8" s="89">
+      <c r="D8" s="76">
         <v>2.667462813169002E-3</v>
       </c>
-      <c r="F8" s="89">
+      <c r="F8" s="76">
         <v>20</v>
       </c>
-      <c r="G8" s="91">
+      <c r="G8" s="78">
         <v>39.700000000000003</v>
       </c>
-      <c r="H8" s="89">
+      <c r="H8" s="76">
         <v>3.9193473830871168E-3</v>
       </c>
-      <c r="J8" s="92">
+      <c r="J8" s="79">
         <v>20</v>
       </c>
-      <c r="K8" s="93">
+      <c r="K8" s="80">
         <v>39.5</v>
       </c>
-      <c r="L8" s="92">
+      <c r="L8" s="79">
         <v>4.4214730756448883E-3</v>
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B9" s="89">
+      <c r="B9" s="76">
         <v>30</v>
       </c>
-      <c r="C9" s="90">
+      <c r="C9" s="77">
         <v>17.633333333333333</v>
       </c>
-      <c r="D9" s="89">
+      <c r="D9" s="76">
         <v>2.5825157175414721E-3</v>
       </c>
-      <c r="F9" s="89">
+      <c r="F9" s="76">
         <v>30</v>
       </c>
-      <c r="G9" s="91">
+      <c r="G9" s="78">
         <v>36.5</v>
       </c>
-      <c r="H9" s="89">
+      <c r="H9" s="76">
         <v>3.9475597396674521E-3</v>
       </c>
-      <c r="J9" s="92">
+      <c r="J9" s="79">
         <v>30</v>
       </c>
-      <c r="K9" s="93">
+      <c r="K9" s="80">
         <v>39.5</v>
       </c>
-      <c r="L9" s="92">
+      <c r="L9" s="79">
         <v>4.3868044297724392E-3</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="89">
+      <c r="B10" s="76">
         <v>40</v>
       </c>
-      <c r="C10" s="90">
+      <c r="C10" s="77">
         <v>15.266666666666666</v>
       </c>
-      <c r="D10" s="89">
+      <c r="D10" s="76">
         <v>2.5716648111675511E-3</v>
       </c>
-      <c r="F10" s="89">
+      <c r="F10" s="76">
         <v>40</v>
       </c>
-      <c r="G10" s="91">
+      <c r="G10" s="78">
         <v>34.799999999999997</v>
       </c>
-      <c r="H10" s="89">
+      <c r="H10" s="76">
         <v>3.9342286261162384E-3</v>
       </c>
-      <c r="J10" s="92">
+      <c r="J10" s="79">
         <v>40</v>
       </c>
-      <c r="K10" s="93">
+      <c r="K10" s="80">
         <v>39.5</v>
       </c>
-      <c r="L10" s="94">
+      <c r="L10" s="79">
         <v>4.3555538194055997E-3</v>
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B11" s="89">
+      <c r="B11" s="76">
         <v>60</v>
       </c>
-      <c r="C11" s="90">
+      <c r="C11" s="77">
         <v>13.166666666666666</v>
       </c>
-      <c r="D11" s="89">
+      <c r="D11" s="76">
         <v>2.5879411707254727E-3</v>
       </c>
-      <c r="F11" s="89">
+      <c r="F11" s="76">
         <v>60</v>
       </c>
-      <c r="G11" s="91">
+      <c r="G11" s="78">
         <v>29.633333333333336</v>
       </c>
-      <c r="H11" s="89">
+      <c r="H11" s="76">
         <v>3.8444761290949239E-3</v>
       </c>
-      <c r="J11" s="92">
+      <c r="J11" s="79">
         <v>60</v>
       </c>
-      <c r="K11" s="93">
+      <c r="K11" s="80">
         <v>32.275000000000006</v>
       </c>
-      <c r="L11" s="92">
+      <c r="L11" s="79">
         <v>4.0267713562129144E-3</v>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B12" s="89">
+      <c r="B12" s="76">
         <v>90</v>
       </c>
-      <c r="C12" s="90">
+      <c r="C12" s="77">
         <v>5.8999999999999995</v>
       </c>
-      <c r="D12" s="89">
+      <c r="D12" s="76">
         <v>2.7266157542214843E-3</v>
       </c>
-      <c r="F12" s="89">
+      <c r="F12" s="76">
         <v>90</v>
       </c>
-      <c r="G12" s="91">
+      <c r="G12" s="78">
         <v>23.400000000000002</v>
       </c>
-      <c r="H12" s="89">
+      <c r="H12" s="76">
         <v>3.2202777397982718E-3</v>
       </c>
-      <c r="J12" s="92">
+      <c r="J12" s="79">
         <v>90</v>
       </c>
-      <c r="K12" s="93">
+      <c r="K12" s="80">
         <v>30.099999999999998</v>
       </c>
-      <c r="L12" s="92">
+      <c r="L12" s="79">
         <v>3.8745870000000001E-3</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B13" s="89">
+      <c r="B13" s="76">
         <v>120</v>
       </c>
-      <c r="C13" s="90">
+      <c r="C13" s="77">
         <v>3.9666666666666663</v>
       </c>
-      <c r="D13" s="89"/>
-      <c r="F13" s="89">
+      <c r="D13" s="76"/>
+      <c r="F13" s="76">
         <v>120</v>
       </c>
-      <c r="G13" s="91">
+      <c r="G13" s="78">
         <v>15.633333333333333</v>
       </c>
-      <c r="H13" s="89">
+      <c r="H13" s="76">
         <v>3.1787730229110855E-3</v>
       </c>
-      <c r="J13" s="92">
+      <c r="J13" s="79">
         <v>120</v>
       </c>
-      <c r="K13" s="93">
+      <c r="K13" s="80">
         <v>24.433333333333334</v>
       </c>
-      <c r="L13" s="95">
+      <c r="L13" s="81">
         <f>AVERAGE(L12,L14)</f>
         <v>3.4375669428413158E-3</v>
       </c>
-      <c r="M13" s="95"/>
+      <c r="M13" s="81"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="F14" s="89">
+      <c r="F14" s="76">
         <v>150</v>
       </c>
-      <c r="G14" s="91">
+      <c r="G14" s="78">
         <v>11.799999999999999</v>
       </c>
-      <c r="H14" s="89"/>
-      <c r="J14" s="92">
+      <c r="H14" s="76"/>
+      <c r="J14" s="79">
         <v>137</v>
       </c>
-      <c r="L14" s="92">
+      <c r="L14" s="79">
         <v>3.0005468856826312E-3</v>
       </c>
-      <c r="M14" s="95">
+      <c r="M14" s="81">
         <v>137</v>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="J15" s="92">
+      <c r="J15" s="79">
         <v>150</v>
       </c>
-      <c r="K15" s="93">
+      <c r="K15" s="80">
         <v>15.933333333333332</v>
       </c>
     </row>

</xml_diff>